<commit_message>
jobs: 2026-09-16 07:56 UTC
</commit_message>
<xml_diff>
--- a/output/jobs.xlsx
+++ b/output/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$M$350</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$M$370</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M350"/>
+  <dimension ref="A1:M370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6230,8 +6230,8 @@
           <t>2026-09-16 15:13:46</t>
         </is>
       </c>
-      <c r="H62" s="4" t="inlineStr"/>
-      <c r="I62" s="4" t="inlineStr"/>
+      <c r="H62" s="4" t="n"/>
+      <c r="I62" s="4" t="n"/>
       <c r="J62" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/social-media-ads-creator-1697016</t>
@@ -6372,8 +6372,8 @@
           <t>2026-09-16 15:06:33</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr"/>
-      <c r="I64" s="4" t="inlineStr"/>
+      <c r="H64" s="4" t="n"/>
+      <c r="I64" s="4" t="n"/>
       <c r="J64" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/bim-lod-500-specialist-1731787</t>
@@ -6445,8 +6445,8 @@
           <t>2026-09-16 15:05:14</t>
         </is>
       </c>
-      <c r="H65" s="4" t="inlineStr"/>
-      <c r="I65" s="4" t="inlineStr"/>
+      <c r="H65" s="4" t="n"/>
+      <c r="I65" s="4" t="n"/>
       <c r="J65" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/cfo-cpa-ca-australian-xero-1731784</t>
@@ -6521,8 +6521,8 @@
           <t>2026-09-16 15:02:34</t>
         </is>
       </c>
-      <c r="H66" s="4" t="inlineStr"/>
-      <c r="I66" s="4" t="inlineStr"/>
+      <c r="H66" s="4" t="n"/>
+      <c r="I66" s="4" t="n"/>
       <c r="J66" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/project-contracts-administrator-1731783</t>
@@ -6675,8 +6675,8 @@
           <t>2026-09-16 15:00:10</t>
         </is>
       </c>
-      <c r="H68" s="4" t="inlineStr"/>
-      <c r="I68" s="4" t="inlineStr"/>
+      <c r="H68" s="4" t="n"/>
+      <c r="I68" s="4" t="n"/>
       <c r="J68" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/wholesale-ecommerce-operations-coordinator-1731781</t>
@@ -6843,8 +6843,8 @@
           <t>2026-09-16 14:59:45</t>
         </is>
       </c>
-      <c r="H69" s="4" t="inlineStr"/>
-      <c r="I69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="n"/>
+      <c r="I69" s="4" t="n"/>
       <c r="J69" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/supply-chain-freight-logistics-coordinator-1731780</t>
@@ -7568,21 +7568,21 @@
           <t>500</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr"/>
-      <c r="F75" s="3" t="inlineStr"/>
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="3" t="n"/>
       <c r="G75" s="3" t="inlineStr">
         <is>
           <t>2026-09-16 14:51:00</t>
         </is>
       </c>
-      <c r="H75" s="4" t="inlineStr"/>
-      <c r="I75" s="4" t="inlineStr"/>
+      <c r="H75" s="4" t="n"/>
+      <c r="I75" s="4" t="n"/>
       <c r="J75" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/6-months-in-france-1731774</t>
         </is>
       </c>
-      <c r="K75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="n"/>
       <c r="L75" s="4" t="inlineStr">
         <is>
           <t>We are looking for a kind, patient, and trustworthy person to live with my old parents in France for six months and help them with their daily routine. Includes Flight, accommodation &amp; food. French &amp; English speaking is required</t>
@@ -8432,8 +8432,8 @@
           <t>2026-09-16 14:40:33</t>
         </is>
       </c>
-      <c r="H83" s="4" t="inlineStr"/>
-      <c r="I83" s="4" t="inlineStr"/>
+      <c r="H83" s="4" t="n"/>
+      <c r="I83" s="4" t="n"/>
       <c r="J83" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/customer-service-support-representative-1731770</t>
@@ -8779,8 +8779,8 @@
           <t>2026-09-16 14:28:00</t>
         </is>
       </c>
-      <c r="H87" s="4" t="inlineStr"/>
-      <c r="I87" s="4" t="inlineStr"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
       <c r="J87" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/executive-assistant-1731763</t>
@@ -8920,21 +8920,21 @@
           <t>14/hr</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr"/>
-      <c r="F88" s="3" t="inlineStr"/>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="3" t="n"/>
       <c r="G88" s="3" t="inlineStr">
         <is>
           <t>2026-09-16 14:27:24</t>
         </is>
       </c>
-      <c r="H88" s="4" t="inlineStr"/>
-      <c r="I88" s="4" t="inlineStr"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
       <c r="J88" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/executive-assistant-1731762</t>
         </is>
       </c>
-      <c r="K88" s="4" t="inlineStr"/>
+      <c r="K88" s="4" t="n"/>
       <c r="L88" s="4" t="inlineStr">
         <is>
           <t>To be considered for this role, please apply directly through our careers page so we can properly review your application. Fill out the application form here: https://morestaffing.careers-page.com/jobs/3c8e4525-b986-47a0-9676-2386d6318b73 Job Title: Executive Assistant Working Hours: Full-Time (40 hours/week) Work Shift: 8:00 AM–4:00…</t>
@@ -8982,8 +8982,8 @@
           <t>2026-09-16 14:23:14</t>
         </is>
       </c>
-      <c r="H89" s="4" t="inlineStr"/>
-      <c r="I89" s="4" t="inlineStr"/>
+      <c r="H89" s="4" t="n"/>
+      <c r="I89" s="4" t="n"/>
       <c r="J89" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/part-time-ghl-meta-ads-specialist-b2c-funnels-1731760</t>
@@ -9961,8 +9961,8 @@
           <t>2026-09-16 14:10:49</t>
         </is>
       </c>
-      <c r="H97" s="4" t="inlineStr"/>
-      <c r="I97" s="4" t="inlineStr"/>
+      <c r="H97" s="4" t="n"/>
+      <c r="I97" s="4" t="n"/>
       <c r="J97" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/ppc-specialist-part-time-position-1731753</t>
@@ -10325,8 +10325,8 @@
           <t>2026-09-16 14:05:50</t>
         </is>
       </c>
-      <c r="H101" s="4" t="inlineStr"/>
-      <c r="I101" s="4" t="inlineStr"/>
+      <c r="H101" s="4" t="n"/>
+      <c r="I101" s="4" t="n"/>
       <c r="J101" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/senior-business-analyst-dayshift-1731752</t>
@@ -10407,8 +10407,8 @@
           <t>2026-09-16 14:04:10</t>
         </is>
       </c>
-      <c r="H102" s="4" t="inlineStr"/>
-      <c r="I102" s="4" t="inlineStr"/>
+      <c r="H102" s="4" t="n"/>
+      <c r="I102" s="4" t="n"/>
       <c r="J102" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/appointment-setter-cold-warm-call-leads-base-10-commission-per-booked-call-1731750</t>
@@ -10480,21 +10480,21 @@
           <t>400</t>
         </is>
       </c>
-      <c r="E103" s="2" t="inlineStr"/>
-      <c r="F103" s="3" t="inlineStr"/>
+      <c r="E103" s="2" t="n"/>
+      <c r="F103" s="3" t="n"/>
       <c r="G103" s="3" t="inlineStr">
         <is>
           <t>2026-09-16 14:01:42</t>
         </is>
       </c>
-      <c r="H103" s="4" t="inlineStr"/>
-      <c r="I103" s="4" t="inlineStr"/>
+      <c r="H103" s="4" t="n"/>
+      <c r="I103" s="4" t="n"/>
       <c r="J103" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/grand-father-sitter-1731748</t>
         </is>
       </c>
-      <c r="K103" s="4" t="inlineStr"/>
+      <c r="K103" s="4" t="n"/>
       <c r="L103" s="4" t="inlineStr">
         <is>
           <t>Live In French Speaking French is necessary Companion and Household Helper – France (6 Months) We are looking for a kind, patient, and trustworthy person to live with my family in France for three months and help them with their…</t>
@@ -11484,8 +11484,8 @@
           <t>2026-09-16 13:43:19</t>
         </is>
       </c>
-      <c r="H113" s="4" t="inlineStr"/>
-      <c r="I113" s="4" t="inlineStr"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
       <c r="J113" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/sales-closing-position-1722822</t>
@@ -11568,8 +11568,8 @@
           <t>2026-09-16 13:43:18</t>
         </is>
       </c>
-      <c r="H114" s="4" t="inlineStr"/>
-      <c r="I114" s="4" t="inlineStr"/>
+      <c r="H114" s="4" t="n"/>
+      <c r="I114" s="4" t="n"/>
       <c r="J114" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/virtual-assistant-wanted-1731741</t>
@@ -11795,8 +11795,8 @@
           <t>2026-09-16 13:39:39</t>
         </is>
       </c>
-      <c r="H116" s="4" t="inlineStr"/>
-      <c r="I116" s="4" t="inlineStr"/>
+      <c r="H116" s="4" t="n"/>
+      <c r="I116" s="4" t="n"/>
       <c r="J116" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/appointment-setter-lead-generation-specialist-1695544</t>
@@ -12002,8 +12002,8 @@
           <t>2026-09-16 13:39:27</t>
         </is>
       </c>
-      <c r="H118" s="4" t="inlineStr"/>
-      <c r="I118" s="4" t="inlineStr"/>
+      <c r="H118" s="4" t="n"/>
+      <c r="I118" s="4" t="n"/>
       <c r="J118" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/amazon-support-ppc-specialist-1715994</t>
@@ -12110,8 +12110,8 @@
           <t>2026-09-16 13:39:26</t>
         </is>
       </c>
-      <c r="H119" s="4" t="inlineStr"/>
-      <c r="I119" s="4" t="inlineStr"/>
+      <c r="H119" s="4" t="n"/>
+      <c r="I119" s="4" t="n"/>
       <c r="J119" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/amazon-ppc-marketplace-specialist-1720485</t>
@@ -12298,21 +12298,21 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="E121" s="2" t="inlineStr"/>
-      <c r="F121" s="3" t="inlineStr"/>
+      <c r="E121" s="2" t="n"/>
+      <c r="F121" s="3" t="n"/>
       <c r="G121" s="3" t="inlineStr">
         <is>
           <t>2026-09-16 13:33:44</t>
         </is>
       </c>
-      <c r="H121" s="4" t="inlineStr"/>
-      <c r="I121" s="4" t="inlineStr"/>
+      <c r="H121" s="4" t="n"/>
+      <c r="I121" s="4" t="n"/>
       <c r="J121" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/senior-full-stack-engineer-next-js-fastapi-ai-b2b-saas-platform-1-500-fixed-milestones-1731736</t>
         </is>
       </c>
-      <c r="K121" s="4" t="inlineStr"/>
+      <c r="K121" s="4" t="n"/>
       <c r="L121" s="4" t="inlineStr">
         <is>
           <t>### About the Project We are building a cutting-edge, autonomous B2B SaaS platform that tracks buying signals, enriches leads, scores buyer intent using LLMs (Claude 3.5 Sonnet / Gemini), and executes autonomous cold outreach. We already have a comprehensive Technical…</t>
@@ -12678,8 +12678,8 @@
           <t>2026-09-16 13:14:42</t>
         </is>
       </c>
-      <c r="H125" s="4" t="inlineStr"/>
-      <c r="I125" s="4" t="inlineStr"/>
+      <c r="H125" s="4" t="n"/>
+      <c r="I125" s="4" t="n"/>
       <c r="J125" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/video-editor-1646088</t>
@@ -12944,8 +12944,8 @@
           <t>800-1000</t>
         </is>
       </c>
-      <c r="E128" s="2" t="inlineStr"/>
-      <c r="F128" s="3" t="inlineStr"/>
+      <c r="E128" s="2" t="n"/>
+      <c r="F128" s="3" t="n"/>
       <c r="G128" s="3" t="inlineStr">
         <is>
           <t>2026-09-16 13:10:14</t>
@@ -12956,13 +12956,13 @@
           <t>Social Media Content Creation, Shopify, Ecommerce</t>
         </is>
       </c>
-      <c r="I128" s="4" t="inlineStr"/>
+      <c r="I128" s="4" t="n"/>
       <c r="J128" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/senior-temu-marketplace-expert-strategic-partner-100k-monthly-profit-goal-1602565</t>
         </is>
       </c>
-      <c r="K128" s="4" t="inlineStr"/>
+      <c r="K128" s="4" t="n"/>
       <c r="L128" s="4" t="inlineStr">
         <is>
           <t>URGENT: I am not looking for an employee. I am looking for a Strategic Partner and a "Growth Shark" to run a high-performance machine. I am Advocate Matan Leker, owner of Leker Projects LLC (US-based). We have built a high-tier…</t>
@@ -12995,8 +12995,8 @@
           <t>600-800</t>
         </is>
       </c>
-      <c r="E129" s="2" t="inlineStr"/>
-      <c r="F129" s="3" t="inlineStr"/>
+      <c r="E129" s="2" t="n"/>
+      <c r="F129" s="3" t="n"/>
       <c r="G129" s="3" t="inlineStr">
         <is>
           <t>2026-09-16 13:10:14</t>
@@ -13007,13 +13007,13 @@
           <t>Marketing, Affiliate Marketing, SEO</t>
         </is>
       </c>
-      <c r="I129" s="4" t="inlineStr"/>
+      <c r="I129" s="4" t="n"/>
       <c r="J129" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/seo-affiliate-operations-manager-gold-ira-niche-attorney-led-us-site-1626519</t>
         </is>
       </c>
-      <c r="K129" s="4" t="inlineStr"/>
+      <c r="K129" s="4" t="n"/>
       <c r="L129" s="4" t="inlineStr">
         <is>
           <t>SEO &amp; Affiliate Operations Manager — Gold IRA Niche (Attorney-Led US Site) Salary: $650/month starting, with clear path to $1,200+/month based on performance Performance Bonus: Up to $200/month additional based on KPIs (traffic, rankings, conversions) Hours: 8 hours/day, Monday to…</t>
@@ -13474,8 +13474,8 @@
           <t>2026-09-16 13:04:53</t>
         </is>
       </c>
-      <c r="H134" s="4" t="inlineStr"/>
-      <c r="I134" s="4" t="inlineStr"/>
+      <c r="H134" s="4" t="n"/>
+      <c r="I134" s="4" t="n"/>
       <c r="J134" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/customer-service-representative-with-project-management-and-marketing-agency-experience-1726547</t>
@@ -14356,8 +14356,8 @@
           <t>2026-09-16 12:48:56</t>
         </is>
       </c>
-      <c r="H143" s="4" t="inlineStr"/>
-      <c r="I143" s="4" t="inlineStr"/>
+      <c r="H143" s="4" t="n"/>
+      <c r="I143" s="4" t="n"/>
       <c r="J143" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/amazon-graphic-designer-packaging-1718687</t>
@@ -15142,8 +15142,8 @@
           <t>2026-09-16 12:40:22</t>
         </is>
       </c>
-      <c r="H150" s="4" t="inlineStr"/>
-      <c r="I150" s="4" t="inlineStr"/>
+      <c r="H150" s="4" t="n"/>
+      <c r="I150" s="4" t="n"/>
       <c r="J150" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/senior-amazon-seo-specialist-affiliate-outreach-1710102</t>
@@ -15233,8 +15233,8 @@
           <t>2026-09-16 12:40:20</t>
         </is>
       </c>
-      <c r="H151" s="4" t="inlineStr"/>
-      <c r="I151" s="4" t="inlineStr"/>
+      <c r="H151" s="4" t="n"/>
+      <c r="I151" s="4" t="n"/>
       <c r="J151" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/amazon-seo-specialist-affiliate-outreach-1678487</t>
@@ -15421,8 +15421,8 @@
           <t>2026-09-16 12:39:53</t>
         </is>
       </c>
-      <c r="H153" s="4" t="inlineStr"/>
-      <c r="I153" s="4" t="inlineStr"/>
+      <c r="H153" s="4" t="n"/>
+      <c r="I153" s="4" t="n"/>
       <c r="J153" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/shopify-web-designer-graphic-designer-1710760</t>
@@ -15959,8 +15959,8 @@
           <t>2026-09-16 12:34:25</t>
         </is>
       </c>
-      <c r="H157" s="4" t="inlineStr"/>
-      <c r="I157" s="4" t="inlineStr"/>
+      <c r="H157" s="4" t="n"/>
+      <c r="I157" s="4" t="n"/>
       <c r="J157" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/work-from-home-administration-assistant-electrical-business-1731714</t>
@@ -17291,8 +17291,8 @@
           <t>$4-$6/hour</t>
         </is>
       </c>
-      <c r="E168" s="2" t="inlineStr"/>
-      <c r="F168" s="3" t="inlineStr"/>
+      <c r="E168" s="2" t="n"/>
+      <c r="F168" s="3" t="n"/>
       <c r="G168" s="3" t="inlineStr">
         <is>
           <t>2026-09-16 12:10:44</t>
@@ -17303,13 +17303,13 @@
           <t>Instagram marketing, Social Media Marketing, Virtual Assistant</t>
         </is>
       </c>
-      <c r="I168" s="4" t="inlineStr"/>
+      <c r="I168" s="4" t="n"/>
       <c r="J168" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/instagram-partnerships-specialist-part-time-1708239</t>
         </is>
       </c>
-      <c r="K168" s="4" t="inlineStr"/>
+      <c r="K168" s="4" t="n"/>
       <c r="L168" s="4" t="inlineStr">
         <is>
           <t>STOP. Read this whole post. Incomplete apps are deleted unread. This is NOT a full-time job. This is NOT SEO, lead-gen agency work, or generic VA admin. If you want 40 hours/week, skip. If your rate is outside $4–$6/hour, skip.…</t>
@@ -18185,8 +18185,8 @@
           <t>2026-09-16 11:48:06</t>
         </is>
       </c>
-      <c r="H177" s="4" t="inlineStr"/>
-      <c r="I177" s="4" t="inlineStr"/>
+      <c r="H177" s="4" t="n"/>
+      <c r="I177" s="4" t="n"/>
       <c r="J177" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/rn-care-operations-coordinator-1731696</t>
@@ -18413,8 +18413,8 @@
           <t>2026-09-16 11:45:14</t>
         </is>
       </c>
-      <c r="H179" s="4" t="inlineStr"/>
-      <c r="I179" s="4" t="inlineStr"/>
+      <c r="H179" s="4" t="n"/>
+      <c r="I179" s="4" t="n"/>
       <c r="J179" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/setters-closers-1704245</t>
@@ -18667,8 +18667,8 @@
           <t>2026-09-16 11:41:01</t>
         </is>
       </c>
-      <c r="H182" s="4" t="inlineStr"/>
-      <c r="I182" s="4" t="inlineStr"/>
+      <c r="H182" s="4" t="n"/>
+      <c r="I182" s="4" t="n"/>
       <c r="J182" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/low-voltage-customer-support-specialist-1707461</t>
@@ -18740,8 +18740,8 @@
           <t>2026-09-16 11:40:23</t>
         </is>
       </c>
-      <c r="H183" s="4" t="inlineStr"/>
-      <c r="I183" s="4" t="inlineStr"/>
+      <c r="H183" s="4" t="n"/>
+      <c r="I183" s="4" t="n"/>
       <c r="J183" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/hiring-now-locksmith-dispatcher-must-have-workiz-experience-1710301</t>
@@ -18816,8 +18816,8 @@
           <t>2026-09-16 11:40:22</t>
         </is>
       </c>
-      <c r="H184" s="4" t="inlineStr"/>
-      <c r="I184" s="4" t="inlineStr"/>
+      <c r="H184" s="4" t="n"/>
+      <c r="I184" s="4" t="n"/>
       <c r="J184" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/need-locksmith-dispatcher-workiz-crm-experience-required-1686154</t>
@@ -18894,8 +18894,8 @@
           <t>2026-09-16 11:40:21</t>
         </is>
       </c>
-      <c r="H185" s="4" t="inlineStr"/>
-      <c r="I185" s="4" t="inlineStr"/>
+      <c r="H185" s="4" t="n"/>
+      <c r="I185" s="4" t="n"/>
       <c r="J185" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/locksmith-dispatcher-wanted-u-s-experience-workiz-required-1686155</t>
@@ -18972,8 +18972,8 @@
           <t>2026-09-16 11:40:20</t>
         </is>
       </c>
-      <c r="H186" s="4" t="inlineStr"/>
-      <c r="I186" s="4" t="inlineStr"/>
+      <c r="H186" s="4" t="n"/>
+      <c r="I186" s="4" t="n"/>
       <c r="J186" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/we-re-hiring-locksmith-dispatcher-secretary-u-s-hvac-company-experience-required-1710274</t>
@@ -19049,8 +19049,8 @@
           <t>2026-09-16 11:40:19</t>
         </is>
       </c>
-      <c r="H187" s="4" t="inlineStr"/>
-      <c r="I187" s="4" t="inlineStr"/>
+      <c r="H187" s="4" t="n"/>
+      <c r="I187" s="4" t="n"/>
       <c r="J187" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/experienced-locksmith-dispatcher-workiz-experience-required-1655831</t>
@@ -19121,8 +19121,8 @@
           <t>2026-09-16 11:40:17</t>
         </is>
       </c>
-      <c r="H188" s="4" t="inlineStr"/>
-      <c r="I188" s="4" t="inlineStr"/>
+      <c r="H188" s="4" t="n"/>
+      <c r="I188" s="4" t="n"/>
       <c r="J188" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/we-re-hiring-experienced-locksmith-dispatcher-workiz-experience-required-1710273</t>
@@ -19198,8 +19198,8 @@
           <t>2026-09-16 11:40:16</t>
         </is>
       </c>
-      <c r="H189" s="4" t="inlineStr"/>
-      <c r="I189" s="4" t="inlineStr"/>
+      <c r="H189" s="4" t="n"/>
+      <c r="I189" s="4" t="n"/>
       <c r="J189" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/we-re-hiring-experienced-chimney-dispatcher-secretary-workiz-experience-required-1710221</t>
@@ -19282,8 +19282,8 @@
           <t>2026-09-16 11:40:15</t>
         </is>
       </c>
-      <c r="H190" s="4" t="inlineStr"/>
-      <c r="I190" s="4" t="inlineStr"/>
+      <c r="H190" s="4" t="n"/>
+      <c r="I190" s="4" t="n"/>
       <c r="J190" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/now-hiring-air-duct-dispatcher-customer-service-workiz-experience-required-1710222</t>
@@ -19367,8 +19367,8 @@
           <t>2026-09-16 11:40:14</t>
         </is>
       </c>
-      <c r="H191" s="4" t="inlineStr"/>
-      <c r="I191" s="4" t="inlineStr"/>
+      <c r="H191" s="4" t="n"/>
+      <c r="I191" s="4" t="n"/>
       <c r="J191" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/experienced-air-duct-dispatcher-workiz-experience-required-1712570</t>
@@ -19449,8 +19449,8 @@
           <t>2026-09-16 11:40:12</t>
         </is>
       </c>
-      <c r="H192" s="4" t="inlineStr"/>
-      <c r="I192" s="4" t="inlineStr"/>
+      <c r="H192" s="4" t="n"/>
+      <c r="I192" s="4" t="n"/>
       <c r="J192" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/air-duct-workiz-crm-experience-required-1712809</t>
@@ -21167,8 +21167,8 @@
           <t>2026-09-16 11:12:20</t>
         </is>
       </c>
-      <c r="H207" s="4" t="inlineStr"/>
-      <c r="I207" s="4" t="inlineStr"/>
+      <c r="H207" s="4" t="n"/>
+      <c r="I207" s="4" t="n"/>
       <c r="J207" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/office-admin-manager-va-remote-work-1731682</t>
@@ -21479,8 +21479,8 @@
           <t>2026-09-16 11:08:29</t>
         </is>
       </c>
-      <c r="H210" s="4" t="inlineStr"/>
-      <c r="I210" s="4" t="inlineStr"/>
+      <c r="H210" s="4" t="n"/>
+      <c r="I210" s="4" t="n"/>
       <c r="J210" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/book-keeper-1731680</t>
@@ -22011,8 +22011,8 @@
           <t>2026-09-16 11:02:21</t>
         </is>
       </c>
-      <c r="H215" s="4" t="inlineStr"/>
-      <c r="I215" s="4" t="inlineStr"/>
+      <c r="H215" s="4" t="n"/>
+      <c r="I215" s="4" t="n"/>
       <c r="J215" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/rpsy-licensed-psychologist-1731677</t>
@@ -23481,8 +23481,8 @@
           <t>2026-09-16 10:40:31</t>
         </is>
       </c>
-      <c r="H229" s="4" t="inlineStr"/>
-      <c r="I229" s="4" t="inlineStr"/>
+      <c r="H229" s="4" t="n"/>
+      <c r="I229" s="4" t="n"/>
       <c r="J229" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/ads-copywriter-wfh-remote-1717774</t>
@@ -23587,8 +23587,8 @@
           <t>2026-09-16 10:38:39</t>
         </is>
       </c>
-      <c r="H230" s="4" t="inlineStr"/>
-      <c r="I230" s="4" t="inlineStr"/>
+      <c r="H230" s="4" t="n"/>
+      <c r="I230" s="4" t="n"/>
       <c r="J230" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/administrative-and-referral-support-assistant-1731666</t>
@@ -24185,8 +24185,8 @@
           <t>2026-09-16 10:32:59</t>
         </is>
       </c>
-      <c r="H234" s="4" t="inlineStr"/>
-      <c r="I234" s="4" t="inlineStr"/>
+      <c r="H234" s="4" t="n"/>
+      <c r="I234" s="4" t="n"/>
       <c r="J234" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/client-support-accountability-coordinator-online-fitness-coaching-business-va-1731656</t>
@@ -24287,8 +24287,8 @@
           <t>2026-09-16 10:32:59</t>
         </is>
       </c>
-      <c r="H235" s="4" t="inlineStr"/>
-      <c r="I235" s="4" t="inlineStr"/>
+      <c r="H235" s="4" t="n"/>
+      <c r="I235" s="4" t="n"/>
       <c r="J235" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/client-support-accountability-coordinator-online-fitness-coaching-business-va-1731660</t>
@@ -24389,8 +24389,8 @@
           <t>2026-09-16 10:32:59</t>
         </is>
       </c>
-      <c r="H236" s="4" t="inlineStr"/>
-      <c r="I236" s="4" t="inlineStr"/>
+      <c r="H236" s="4" t="n"/>
+      <c r="I236" s="4" t="n"/>
       <c r="J236" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/client-support-accountability-coordinator-online-fitness-coaching-business-va-1731661</t>
@@ -24691,8 +24691,8 @@
           <t>2026-09-16 10:25:10</t>
         </is>
       </c>
-      <c r="H239" s="4" t="inlineStr"/>
-      <c r="I239" s="4" t="inlineStr"/>
+      <c r="H239" s="4" t="n"/>
+      <c r="I239" s="4" t="n"/>
       <c r="J239" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/creative-strategist-copywriter-1731657</t>
@@ -25023,8 +25023,8 @@
           <t>2026-09-16 10:19:53</t>
         </is>
       </c>
-      <c r="H242" s="4" t="inlineStr"/>
-      <c r="I242" s="4" t="inlineStr"/>
+      <c r="H242" s="4" t="n"/>
+      <c r="I242" s="4" t="n"/>
       <c r="J242" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/direct-response-copywriter-1654158</t>
@@ -25385,8 +25385,8 @@
           <t>2026-09-16 10:14:46</t>
         </is>
       </c>
-      <c r="H245" s="4" t="inlineStr"/>
-      <c r="I245" s="4" t="inlineStr"/>
+      <c r="H245" s="4" t="n"/>
+      <c r="I245" s="4" t="n"/>
       <c r="J245" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/virtual-assistant-general-merchandise-listings-ebay-1731654</t>
@@ -26016,8 +26016,8 @@
           <t>2026-09-16 10:01:58</t>
         </is>
       </c>
-      <c r="H250" s="4" t="inlineStr"/>
-      <c r="I250" s="4" t="inlineStr"/>
+      <c r="H250" s="4" t="n"/>
+      <c r="I250" s="4" t="n"/>
       <c r="J250" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/social-media-marketing-strategist-no-editing-required-1731646</t>
@@ -26585,8 +26585,8 @@
           <t>2026-09-16 10:00:06</t>
         </is>
       </c>
-      <c r="H254" s="4" t="inlineStr"/>
-      <c r="I254" s="4" t="inlineStr"/>
+      <c r="H254" s="4" t="n"/>
+      <c r="I254" s="4" t="n"/>
       <c r="J254" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/remote-front-desk-operations-coordinator-1721664</t>
@@ -26759,8 +26759,8 @@
           <t>2026-09-16 10:00:04</t>
         </is>
       </c>
-      <c r="H255" s="4" t="inlineStr"/>
-      <c r="I255" s="4" t="inlineStr"/>
+      <c r="H255" s="4" t="n"/>
+      <c r="I255" s="4" t="n"/>
       <c r="J255" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/virtual-practice-and-social-media-assistant-australia-clinical-psychology-practice-1730408</t>
@@ -26865,8 +26865,8 @@
           <t>2026-09-16 10:00:04</t>
         </is>
       </c>
-      <c r="H256" s="4" t="inlineStr"/>
-      <c r="I256" s="4" t="inlineStr"/>
+      <c r="H256" s="4" t="n"/>
+      <c r="I256" s="4" t="n"/>
       <c r="J256" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/virtual-assistnce-work-from-home-1730667</t>
@@ -27346,8 +27346,8 @@
           <t>2026-09-16 10:00:03</t>
         </is>
       </c>
-      <c r="H261" s="4" t="inlineStr"/>
-      <c r="I261" s="4" t="inlineStr"/>
+      <c r="H261" s="4" t="n"/>
+      <c r="I261" s="4" t="n"/>
       <c r="J261" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/ophthalmology-surgical-coordinator-remote-1730368</t>
@@ -27459,8 +27459,8 @@
           <t>2026-09-16 10:00:03</t>
         </is>
       </c>
-      <c r="H262" s="4" t="inlineStr"/>
-      <c r="I262" s="4" t="inlineStr"/>
+      <c r="H262" s="4" t="n"/>
+      <c r="I262" s="4" t="n"/>
       <c r="J262" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/car-rental-business-operations-1731166</t>
@@ -27575,8 +27575,8 @@
           <t>2026-09-16 10:00:02</t>
         </is>
       </c>
-      <c r="H263" s="4" t="inlineStr"/>
-      <c r="I263" s="4" t="inlineStr"/>
+      <c r="H263" s="4" t="n"/>
+      <c r="I263" s="4" t="n"/>
       <c r="J263" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/assistant-designer-for-bathrooms-1622437</t>
@@ -27760,8 +27760,8 @@
           <t>2026-09-16 10:00:02</t>
         </is>
       </c>
-      <c r="H265" s="4" t="inlineStr"/>
-      <c r="I265" s="4" t="inlineStr"/>
+      <c r="H265" s="4" t="n"/>
+      <c r="I265" s="4" t="n"/>
       <c r="J265" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/email-marketing-specialist-1714234</t>
@@ -27927,8 +27927,8 @@
           <t>2026-09-16 10:00:02</t>
         </is>
       </c>
-      <c r="H266" s="4" t="inlineStr"/>
-      <c r="I266" s="4" t="inlineStr"/>
+      <c r="H266" s="4" t="n"/>
+      <c r="I266" s="4" t="n"/>
       <c r="J266" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/math-tutor-1729631</t>
@@ -27986,8 +27986,8 @@
           <t>2026-09-16 10:00:02</t>
         </is>
       </c>
-      <c r="H267" s="4" t="inlineStr"/>
-      <c r="I267" s="4" t="inlineStr"/>
+      <c r="H267" s="4" t="n"/>
+      <c r="I267" s="4" t="n"/>
       <c r="J267" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/youtube-ai-script-writer-ai-voiceover-generation-animals-creatures-long-term-1731442</t>
@@ -28150,8 +28150,8 @@
           <t>2026-09-16 10:00:01</t>
         </is>
       </c>
-      <c r="H269" s="4" t="inlineStr"/>
-      <c r="I269" s="4" t="inlineStr"/>
+      <c r="H269" s="4" t="n"/>
+      <c r="I269" s="4" t="n"/>
       <c r="J269" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/sales-business-development-specialist-1713906</t>
@@ -29125,8 +29125,8 @@
           <t>2026-09-16 09:43:03</t>
         </is>
       </c>
-      <c r="H277" s="4" t="inlineStr"/>
-      <c r="I277" s="4" t="inlineStr"/>
+      <c r="H277" s="4" t="n"/>
+      <c r="I277" s="4" t="n"/>
       <c r="J277" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/admin-va-job-tracking-data-accuracy-trade-construction-experience-non-negotiable-1731640</t>
@@ -29243,8 +29243,8 @@
           <t>2026-09-16 09:41:41</t>
         </is>
       </c>
-      <c r="H278" s="4" t="inlineStr"/>
-      <c r="I278" s="4" t="inlineStr"/>
+      <c r="H278" s="4" t="n"/>
+      <c r="I278" s="4" t="n"/>
       <c r="J278" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/tiktok-organic-creator-1731639</t>
@@ -29475,8 +29475,8 @@
           <t>2026-09-16 09:41:22</t>
         </is>
       </c>
-      <c r="H280" s="4" t="inlineStr"/>
-      <c r="I280" s="4" t="inlineStr"/>
+      <c r="H280" s="4" t="n"/>
+      <c r="I280" s="4" t="n"/>
       <c r="J280" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/tiktok-creator-1731638</t>
@@ -29699,8 +29699,8 @@
           <t>2026-09-16 09:40:24</t>
         </is>
       </c>
-      <c r="H282" s="4" t="inlineStr"/>
-      <c r="I282" s="4" t="inlineStr"/>
+      <c r="H282" s="4" t="n"/>
+      <c r="I282" s="4" t="n"/>
       <c r="J282" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/tiktok-ai-editor-1731636</t>
@@ -29923,8 +29923,8 @@
           <t>2026-09-16 09:39:27</t>
         </is>
       </c>
-      <c r="H284" s="4" t="inlineStr"/>
-      <c r="I284" s="4" t="inlineStr"/>
+      <c r="H284" s="4" t="n"/>
+      <c r="I284" s="4" t="n"/>
       <c r="J284" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/organic-tiktok-content-1731634</t>
@@ -30730,8 +30730,8 @@
           <t>2026-09-16 09:33:55</t>
         </is>
       </c>
-      <c r="H291" s="4" t="inlineStr"/>
-      <c r="I291" s="4" t="inlineStr"/>
+      <c r="H291" s="4" t="n"/>
+      <c r="I291" s="4" t="n"/>
       <c r="J291" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/property-manager-short-rentals-1731628</t>
@@ -31268,8 +31268,8 @@
           <t>2026-09-16 09:28:34</t>
         </is>
       </c>
-      <c r="H294" s="4" t="inlineStr"/>
-      <c r="I294" s="4" t="inlineStr"/>
+      <c r="H294" s="4" t="n"/>
+      <c r="I294" s="4" t="n"/>
       <c r="J294" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/senior-australian-public-practice-bookkeeper-remote-independent-contractor-philippines-1724637</t>
@@ -31718,8 +31718,8 @@
           <t>2026-09-16 09:21:18</t>
         </is>
       </c>
-      <c r="H297" s="4" t="inlineStr"/>
-      <c r="I297" s="4" t="inlineStr"/>
+      <c r="H297" s="4" t="n"/>
+      <c r="I297" s="4" t="n"/>
       <c r="J297" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/full-time-outbound-calling-live-transfers-medicare-us-daytime-hours-1719284</t>
@@ -32190,8 +32190,8 @@
           <t>2026-09-16 09:17:23</t>
         </is>
       </c>
-      <c r="H301" s="4" t="inlineStr"/>
-      <c r="I301" s="4" t="inlineStr"/>
+      <c r="H301" s="4" t="n"/>
+      <c r="I301" s="4" t="n"/>
       <c r="J301" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/digital-platform-sales-specialist-1731618</t>
@@ -32797,8 +32797,8 @@
           <t>2026-09-16 09:04:11</t>
         </is>
       </c>
-      <c r="H307" s="4" t="inlineStr"/>
-      <c r="I307" s="4" t="inlineStr"/>
+      <c r="H307" s="4" t="n"/>
+      <c r="I307" s="4" t="n"/>
       <c r="J307" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/amazon-seo-manager-1703028</t>
@@ -33415,8 +33415,8 @@
           <t>2026-09-16 08:56:26</t>
         </is>
       </c>
-      <c r="H313" s="4" t="inlineStr"/>
-      <c r="I313" s="4" t="inlineStr"/>
+      <c r="H313" s="4" t="n"/>
+      <c r="I313" s="4" t="n"/>
       <c r="J313" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/appointment-setter-gold-silver-industry-1731605</t>
@@ -33831,8 +33831,8 @@
           <t>2026-09-16 08:50:45</t>
         </is>
       </c>
-      <c r="H318" s="4" t="inlineStr"/>
-      <c r="I318" s="4" t="inlineStr"/>
+      <c r="H318" s="4" t="n"/>
+      <c r="I318" s="4" t="n"/>
       <c r="J318" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/animal-animation-1686925</t>
@@ -33905,8 +33905,8 @@
           <t>2026-09-16 08:50:38</t>
         </is>
       </c>
-      <c r="H319" s="4" t="inlineStr"/>
-      <c r="I319" s="4" t="inlineStr"/>
+      <c r="H319" s="4" t="n"/>
+      <c r="I319" s="4" t="n"/>
       <c r="J319" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/video-animator-everything-professor-1725590</t>
@@ -33981,8 +33981,8 @@
           <t>2026-09-16 08:49:31</t>
         </is>
       </c>
-      <c r="H320" s="4" t="inlineStr"/>
-      <c r="I320" s="4" t="inlineStr"/>
+      <c r="H320" s="4" t="n"/>
+      <c r="I320" s="4" t="n"/>
       <c r="J320" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/virtual-receptionist-va-remote-fast-hiring-24-hour-review-1641955</t>
@@ -34217,8 +34217,8 @@
           <t>2026-09-16 08:48:32</t>
         </is>
       </c>
-      <c r="H322" s="4" t="inlineStr"/>
-      <c r="I322" s="4" t="inlineStr"/>
+      <c r="H322" s="4" t="n"/>
+      <c r="I322" s="4" t="n"/>
       <c r="J322" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/social-media-coordinator-1731600</t>
@@ -34316,8 +34316,8 @@
           <t>2026-09-16 08:47:47</t>
         </is>
       </c>
-      <c r="H323" s="4" t="inlineStr"/>
-      <c r="I323" s="4" t="inlineStr"/>
+      <c r="H323" s="4" t="n"/>
+      <c r="I323" s="4" t="n"/>
       <c r="J323" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/client-video-production-coordinator-philippines-only-1716165</t>
@@ -34565,8 +34565,8 @@
           <t>2026-09-16 08:43:01</t>
         </is>
       </c>
-      <c r="H325" s="4" t="inlineStr"/>
-      <c r="I325" s="4" t="inlineStr"/>
+      <c r="H325" s="4" t="n"/>
+      <c r="I325" s="4" t="n"/>
       <c r="J325" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/video-editor-b2b-marketing-1696784</t>
@@ -35592,8 +35592,8 @@
           <t>2026-09-16 08:34:49</t>
         </is>
       </c>
-      <c r="H334" s="4" t="inlineStr"/>
-      <c r="I334" s="4" t="inlineStr"/>
+      <c r="H334" s="4" t="n"/>
+      <c r="I334" s="4" t="n"/>
       <c r="J334" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/tarot-reader-1697745</t>
@@ -35707,8 +35707,8 @@
           <t>2026-09-16 08:32:12</t>
         </is>
       </c>
-      <c r="H335" s="4" t="inlineStr"/>
-      <c r="I335" s="4" t="inlineStr"/>
+      <c r="H335" s="4" t="n"/>
+      <c r="I335" s="4" t="n"/>
       <c r="J335" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/merchant-support-officer-payment-service-provider-1685398</t>
@@ -35798,8 +35798,8 @@
           <t>2026-09-16 08:29:30</t>
         </is>
       </c>
-      <c r="H336" s="4" t="inlineStr"/>
-      <c r="I336" s="4" t="inlineStr"/>
+      <c r="H336" s="4" t="n"/>
+      <c r="I336" s="4" t="n"/>
       <c r="J336" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/influencer-marketing-specialist-1731587</t>
@@ -35907,8 +35907,8 @@
           <t>2026-09-16 08:26:01</t>
         </is>
       </c>
-      <c r="H337" s="4" t="inlineStr"/>
-      <c r="I337" s="4" t="inlineStr"/>
+      <c r="H337" s="4" t="n"/>
+      <c r="I337" s="4" t="n"/>
       <c r="J337" s="5" t="inlineStr">
         <is>
           <t>https://www.onlinejobs.ph/jobseekers/job/real-estate-transaction-coordinator-california-1731585</t>
@@ -37631,8 +37631,1729 @@
         </is>
       </c>
     </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>1731817</t>
+        </is>
+      </c>
+      <c r="B351" s="3" t="inlineStr">
+        <is>
+          <t>General Virtual Assistant – Research, Admin, and Operations Support</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="D351" s="3" t="inlineStr">
+        <is>
+          <t>$268.00</t>
+        </is>
+      </c>
+      <c r="E351" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F351" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G351" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:52:18</t>
+        </is>
+      </c>
+      <c r="H351" s="4" t="inlineStr">
+        <is>
+          <t>Market Research, Business development, Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="I351" s="4" t="inlineStr">
+        <is>
+          <t>Market Research, Business development, Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="J351" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/general-virtual-assistant-research-admin-and-operations-support-1731817</t>
+        </is>
+      </c>
+      <c r="K351" s="4" t="inlineStr">
+        <is>
+          <t>We are looking for a sharp and reliable General Virtual Assistant to support a growing company with research, business operations, task coordination, and general administrative work.
+This role is ideal for someone who is organized, curious, detail-oriented, and able to help turn information into clear next steps. You should be comfortable researching online, organizing findings, supporting internal tasks, and helping keep daily work moving.
+You may help with:
+Online research on companies, tools, services, ideas, and business topics
+Organizing research into clear summaries, lists, or spreadsheets
+Supporting business operations by helping track information, updates, and next steps
+Assisting with assigned tasks, follow-ups, and small projects
+Updating documents, trackers, and online records
+Handling general admin tasks as needed
+We are looking for someone who:
+Writes clearly and professionally
+Pays attention to detail
+Can research and summarize information well
+Is comfortable using Google Docs, Google Sheets, Gmail, and online tools
+Can follow instructions and ask good questions
+Is dependable, organized, and willing to learn
+To apply, please share your experience, the tools you have used, and one example of work you have done involving research, admin support, or task coordination.
+Important: At the very top of your application, write the word CLARITY.</t>
+        </is>
+      </c>
+      <c r="L351" s="4" t="inlineStr">
+        <is>
+          <t>We are looking for a sharp and reliable General Virtual Assistant to support a growing company with research, business operations, task coordination, and general administrative work. This role is ideal for someone who is organized, curious, detail-oriented, and able to…</t>
+        </is>
+      </c>
+      <c r="M351" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>1731815</t>
+        </is>
+      </c>
+      <c r="B352" s="3" t="inlineStr">
+        <is>
+          <t>Facebook Ads Specialist – Full-Time, Long-Term</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D352" s="3" t="inlineStr">
+        <is>
+          <t>$5/ hour</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F352" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G352" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:50:26</t>
+        </is>
+      </c>
+      <c r="H352" s="4" t="inlineStr">
+        <is>
+          <t>Meta Pixel, Facebook Ads, Ads Management</t>
+        </is>
+      </c>
+      <c r="I352" s="4" t="inlineStr">
+        <is>
+          <t>Meta Pixel, Facebook Ads, Ads Management</t>
+        </is>
+      </c>
+      <c r="J352" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/facebook-ads-specialist-full-time-long-term-1731815</t>
+        </is>
+      </c>
+      <c r="K352" s="4" t="inlineStr">
+        <is>
+          <t>---------- 
+ Simplified is hiring a
+ Facebook
+ Ads specialist. We're a US-based online education company that helps students prepare for the MCAT (the medical school entrance exam). Paid ads are our main way of reaching new students, and we're looking for someone to own our
+ Facebook
+ ads long-term.
+WHAT YOU'LL DO
+- Set up, run, and improve
+ Facebook
+ and Instagram ad campaigns
+- Test new ads (hooks, images, videos) and tell us what's working
+- Write ad copy and give simple direction to our designer/video editor
+- Keep tracking set up correctly (Pixel, Conversions API, UTMs)
+- Send a short daily update and a weekly results report
+WHAT WE'RE LOOKING FOR
+- At least 1–2 years running
+ Facebook
+ ads for a business or clients
+- Lead generation experience (getting sign-ups, bookings, or inquiries)
+- Comfortable using Ads Manager, Business Manager, and Events Manager
+- Good written English, and you speak up when something looks off
+- Reliable internet and able to overlap a few hours with US Pacific Time
+NICE TO HAVE (NOT REQUIRED)
+- Ads for courses, coaching, or education
+- Google Ads or YouTube Ads
+- GoHighLevel, ClickFunnels, or similar tools
+PAY &amp; DETAILS
+- $800–$1,200/month depending on experience
+- Full-time, 40 hours/week
+- Long-term role with raises based on results
+HOW TO APPLY
+Start your message with the word "PIXEL" and tell us:
+1. How long you'
+ ---------- 
+ run
+ Facebook
+ ads and the biggest monthly budget you've managed
+2. What kinds of businesses you've run ads for
+3. One result you're proud of (a screenshot is great, and you can hide client names)
+Shortlisted applicants will be invited to a short video call.</t>
+        </is>
+      </c>
+      <c r="L352" s="4" t="inlineStr">
+        <is>
+          <t>MCAT Simplified is hiring a Facebook Ads specialist. We're a US-based online education company that helps students prepare for the MCAT (the medical school entrance exam). Paid ads are our main way of reaching new students, and we're looking for…</t>
+        </is>
+      </c>
+      <c r="M352" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>1698611</t>
+        </is>
+      </c>
+      <c r="B353" s="3" t="inlineStr">
+        <is>
+          <t>Social Media Strategist &amp; Growth Manager</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D353" s="3" t="inlineStr">
+        <is>
+          <t>$5-10/hr</t>
+        </is>
+      </c>
+      <c r="E353" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F353" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G353" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:50:05</t>
+        </is>
+      </c>
+      <c r="H353" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Content Creation, Social Media Management, PPC</t>
+        </is>
+      </c>
+      <c r="I353" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Content Creation, Social Media Management, PPC</t>
+        </is>
+      </c>
+      <c r="J353" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/social-media-strategist-growth-manager-1698611</t>
+        </is>
+      </c>
+      <c r="K353" s="4" t="inlineStr">
+        <is>
+          <t>We're looking for an experienced Social Media Strategist &amp; Growth Manager to take ownership of our brands' social media presence.
+This is not a content posting role. We're looking for someone who can develop strategy, execute it, and continuously optimize performance across multiple social media platforms. Depending on your skills, you'll personally create content where appropriate and coordinate with designers or other tea
+ ---------- 
+mbers when required.
+The ideal candidate understands how social media algorithms work, knows how to build engaged communities, and can translate business objectives into measurable social media growth.
+Key Responsibilities
+Develop and execute social media strategies across Instagram,
+ Facebook
+, TikTok, and other relevant platforms.
+Plan and manage content calendars aligned with business objectives.
+Create and publish engaging content, including captions, graphics, and short-form videos where appropriate.
+Grow audience reach, engagement, and brand awareness through organic strategies.
+Monitor platform performance and continuously improve results using data and insights.
+Engage with followers by responding to comments, messages, and community interactions.
+Stay up to date with platform updates, trends, and best practices.
+Coordinate with designers, content creators, and marketing tea
+ ---------- 
+mbers when required.
+Required Experience
+Minimum 2 years' hands-on experience managing business social media accounts.
+Strong understanding of Instagram,
+ Facebook
+, and TikTok algorithms.
+Proven experience developing and implementing successful social media strategies.
+Strong copywriting and communication skills.
+Experience with Meta Business Suite and social media analytics.
+Ability to work independently while managing multiple priorities.
+Bonus Skills
+Experience with eCommerce brands.
+Canva or basic graphic design.
+Short-form video editing.
+Paid social advertising.
+Experience working with Australian businesses.
+Work Setup
+Remote position.
+Part-time initially with the opportunity to expand.
+Stable internet and power connection are essential.
+During allocated working hours, your focus should be fully dedicated to our projects.
+Application Requirements
+Please submit:
+-Your resume.
+-A short introduction highlighting your relevant experience.
+-Links to 3-5 social media accounts or campaigns you have personally managed.
+-Examples of content you have created.
+-Your expected hourly rate.
+-The completed Self-Assessment Checklist below.
+-A short video (maximum 3 minutes) introducing yourself. In your video, briefly explain:
+Your social media background.
+The strategies you've implemented to grow accounts.
+Your personal role in previous projects.
+Why you're a good fit for this position.
+Please upload your video to Google Drive, Dropbox, OneDrive, or a similar platform, ensure the link is publicly accessible (no password or permission request), and include the link in your application.
+Applications submitted without both the completed Self-Assessment Checklist and the video introduction will not be reviewed.
+Social Media Self-Assessment
+Please rate yourself as None, Basic, or Professional.
+Strategy &amp; Growth
+Social media strategy development
+Organic account growth
+Content planning
+Community building
+Performance analysis
+Trend research and implementation
+Platforms
+Instagram
+Facebook
+TikTok
+LinkedIn
+YouTube Shorts (optional)
+Content
+Copywriting
+Content calendars
+Canva
+Short-form video creation/editing
+Storytelling and brand voice
+Tools
+Meta Business Suite
+TikTok Analytics
+Google Analytics
+Scheduling tools (Buffer, Later, Metricool, etc.)
+Google Docs/Sheets
+Experience Summary
+Years of social media experience
+Industries worked with
+eCommerce experience (Yes/No)
+Please provide 3-5 portfolio links
+Only shortlisted candidates will be invited to interview. During the interview, we'll discuss your previous work in detail, including your strategy, execution, and the measurable results you achieved.
+Important Note:
+During the interview process, we may ask you to share and walk us through examples of recent work you have completed for previous clients or projects. This helps us better understand your approach, strategy, decision-making, and the quality of your work. If you're unable or unwilling to discuss or demonstrate examples of your recent work for any reason, this role is unlikely to be a good fit.</t>
+        </is>
+      </c>
+      <c r="L353" s="4" t="inlineStr">
+        <is>
+          <t>We're looking for an experienced Social Media Strategist &amp; Growth Manager to take ownership of our brands' social media presence. This is not a content posting role. We're looking for someone who can develop strategy, execute it, and continuously optimize…</t>
+        </is>
+      </c>
+      <c r="M353" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>1731814</t>
+        </is>
+      </c>
+      <c r="B354" s="3" t="inlineStr">
+        <is>
+          <t>Remote Virtual Assistant – Business Support and Online Tasks</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="D354" s="3" t="inlineStr">
+        <is>
+          <t>$268.00</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F354" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G354" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:49:52</t>
+        </is>
+      </c>
+      <c r="H354" s="4" t="inlineStr">
+        <is>
+          <t>Business development, Operation Management, Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="I354" s="4" t="inlineStr">
+        <is>
+          <t>Business development, Operation Management, Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="J354" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/remote-virtual-assistant-business-support-and-online-tasks-1731814</t>
+        </is>
+      </c>
+      <c r="K354" s="4" t="inlineStr">
+        <is>
+          <t>We are hiring a Remote Virtual Assistant to help with business support, online research, task management, and general administrative duties.
+The right person should be able to work through different types of assignments, organize information clearly, and help support ongoing company needs. This role requires someone who can stay focused, communicate well, and complete work with care.
+Responsibilities may include:
+Researching information online and presenting useful findings
+Assisting with business operations tasks such as tracking updates, organizing details, and supporting internal processes
+Helping manage task lists, follow-up items, and project notes
+Preparing simple summaries, comparisons, checklists, or documents
+Updating spreadsheets, folders, records, and shared files
+Completing general admin assignments as needed
+A strong candidate will be:
+Organized and detail-oriented
+Comfortable with online research
+Able to write clear summaries and updates
+Good at following instructions and meeting deadlines
+Comfortable using Google Workspace and similar tools
+Able to work independently while keeping communication clear
+Flexible and willing to support different areas of the business
+To apply, please send a short message explaining your relevant experience, your availability, and why you would be a strong fit for this type of VA role.
+At the very top of your application, write the word FOCUS.</t>
+        </is>
+      </c>
+      <c r="L354" s="4" t="inlineStr">
+        <is>
+          <t>We are hiring a Remote Virtual Assistant to help with business support, online research, task management, and general administrative duties. The right person should be able to work through different types of assignments, organize information clearly, and help support ongoing…</t>
+        </is>
+      </c>
+      <c r="M354" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>1433117</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>SEO Expert</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="D355" s="3" t="inlineStr">
+        <is>
+          <t>$8 - $12+ per hour</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F355" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G355" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:40:11</t>
+        </is>
+      </c>
+      <c r="H355" s="4" t="inlineStr">
+        <is>
+          <t>Local SEO, SEO Analysis, Content Management</t>
+        </is>
+      </c>
+      <c r="I355" s="4" t="inlineStr">
+        <is>
+          <t>Local SEO, SEO Analysis, Content Management</t>
+        </is>
+      </c>
+      <c r="J355" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/seo-expert-1433117</t>
+        </is>
+      </c>
+      <c r="K355" s="4" t="inlineStr">
+        <is>
+          <t>Summary
+We need someone who will act as our expert consultant for our Automotive SEO company. You will only provide guidance, recommendations or advice. You need to be available for meetings during US Eastern or Pacific business hours.
+The person we are looking for needs to:
+- Speak and write English fluently or almost native as this role will require you to present and talk to executives during meetings
+- Know white-hat SEO strategies and be able to develop a plan on how to increase a dealership's organic traffic, conversions, and search result rankings
+- Work with the development team to ensure SEO best practices are properly implemented on newly developed code
+- Recommend changes to website architecture, content, linking and other factors to improve SEO positions for target keywords
+- Update/Create reports and charts for presentations
+- Be able to do content, page or site audits and provide recommendations to optimize content and improve search result rankings
+- Be our go-to person for any questions or concerns regarding SEO best practices
+- Be able to provide examples of success from previous work
+- Be able to assist the Project Manager with recommendations or advice for any content creation, programming, and analysis related to SEO to successfully complete tasks and projects
+Requirements and skills:
+- Proven SEO experience
+- Solid understanding of performance marketing, conversion, and online customer acquisition
+- In-depth experience with website analytics tools (e.g, Google Analytics, Google Search Console, SEMRush, Adobe Analytics)
+- Experience with A/B and multivariate experiments
+- Working knowledge of HTML, CSS, and JavaScript development and constraints
+- Knowledge of ranking factors and search engine algorithms
+- Up-to-date with the latest trends and best practices in SEO and SEM
+- Knowledge of keyword research and data mining tools
+- Able to complete competitive analysis of other companies within the industry
+- Familiarity with WordPress or other content management systems</t>
+        </is>
+      </c>
+      <c r="L355" s="4" t="inlineStr">
+        <is>
+          <t>Summary We need someone who will act as our expert consultant for our Automotive SEO company. You will only provide guidance, recommendations or advice. You need to be available for meetings during US Eastern or Pacific business hours. The person…</t>
+        </is>
+      </c>
+      <c r="M355" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>1731812</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>Social Media Content Uploader – No Filming or Editing (IG, YouTube, FB)</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="D356" s="3" t="inlineStr">
+        <is>
+          <t>from $3 to $7 per hour</t>
+        </is>
+      </c>
+      <c r="E356" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F356" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G356" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:39:00</t>
+        </is>
+      </c>
+      <c r="H356" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Management, Instagram marketing, Youtube Marketing</t>
+        </is>
+      </c>
+      <c r="I356" s="4" t="inlineStr">
+        <is>
+          <t>Social Media Management, Instagram marketing, Youtube Marketing</t>
+        </is>
+      </c>
+      <c r="J356" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/social-media-content-uploader-no-filming-or-editing-ig-youtube-fb-1731812</t>
+        </is>
+      </c>
+      <c r="K356" s="4" t="inlineStr">
+        <is>
+          <t>We’re a fast-growing company with 12M+ users looking for reliable people to help us upload ready-made social media content.
+This is a simple side job you can do in your free time.
+You do not need to film, edit, write captions, or create content. We provide the videos and descriptions.
+What you’ll do
+Every day, you’ll receive 2 ready-made videos.
+You must upload both videos to:
+- Instagram
+- YouTube
+-
+ Facebook
+That means:
+2 videos × 3 platforms = 6 uploads per day
+The most important thing is consistency. You must be able to post every day.
+The work only takes a few minutes per day and can be done at a time that works for you.
+Pay:
+$45/month (Paid every 2 weeks): $0.25 per upload
+Extra bonuses based on video performance and views
+Bonuses can reach up to $100 for a single top-performing video
+Paid Testing Phase
+There is a short paid testing phase first.
+You will receive $5 for completing the test correctly.
+Requirements
+- Reliable smartphone
+- Stable internet connection
+- Able to post every day
+- Good attention to detail
+- Able to follow simple step-by-step instructions
+- Reliable and independent
+This is a good fit if you’re looking for a simple, flexible side job that you can do alongside school, another job, or other responsibilities.
+Send DM and you'll get instructions how to start!</t>
+        </is>
+      </c>
+      <c r="L356" s="4" t="inlineStr">
+        <is>
+          <t>We’re a fast-growing company with 12M+ users looking for reliable people to help us upload ready-made social media content. This is a simple side job you can do in your free time. You do not need to film, edit, write…</t>
+        </is>
+      </c>
+      <c r="M356" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>1731811</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="inlineStr">
+        <is>
+          <t>Amazon PPC and Listing Specialist for Amazon.de (Part-time, 10h/week, long-term)</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="D357" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F357" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G357" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:38:47</t>
+        </is>
+      </c>
+      <c r="H357" s="4" t="inlineStr">
+        <is>
+          <t>Amazon, Seller Central, Amazon PPC</t>
+        </is>
+      </c>
+      <c r="I357" s="4" t="inlineStr">
+        <is>
+          <t>Amazon, Seller Central, Amazon PPC</t>
+        </is>
+      </c>
+      <c r="J357" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/amazon-ppc-and-listing-specialist-for-amazon-de-part-time-10h-week-long-term-1731811</t>
+        </is>
+      </c>
+      <c r="K357" s="4" t="inlineStr">
+        <is>
+          <t>We are a German dietary supplement brand (vitamins, minerals, capsules) selling on 
+ ---------- 
+. The account is run by the founder, and we want one person who takes ownership of Amazon Germany: ads, listings, account health, and the rules that come with supplements.
+YOUR JOB
+- PPC: build and manage Sponsored Products, Sponsored Brands and Sponsored Display. German keyword research, bids, negatives, budgets, weekly optimization. Targets: profitable ACoS, growing organic rank, more repeat buyers via Subscribe &amp; Save
+- Listings: titles, bullets, backend keywords, A+ content and images. Copy is German, we provide translations and product facts, you provide structure, keyword logic and conversion thinking
+- Compliance: you know that supplements on 
+ ---------- 
+ have strict rules. No health or healing claims (EU Health Claims Regulation 1924/2006), only approved claims, correct dosage and warning texts, restricted keywords in ads. You check every listing and every ad against these rules before it goes live, and you tell us when Amazon changes something
+- Account health: Buy Box, inventory (FBA), suppressed or blocked listings, category approvals, Seller Support cases, reviews and Vine
+- Reporting: one short weekly Google Sheet: ad spend, sales, ACoS, TACoS, organic vs paid, Subscribe &amp; Save share, rank of our top products, what you changed and why
+- Competitors: watch the other supplement sellers in our categories and report price, listing and ad changes
+WHAT WE EXPECT
+- At least 2 years hands-on in Amazon Seller Central and Amazon Ads, ideally with supplements, health or beauty products on a European marketplace (DE, FR, IT, ES or UK)
+- You can show accounts you managed with spend, ACoS and sales growth (screenshots, client names blurred is fine)
+- You have dealt with restricted categories, listing suppressions or claim rejections before and can describe how you solved them
+- Helium 10, Jungle Scout, DataDive or similar for German keyword research (you dont need to speak German, we check language, you check data). Basic German reading is a plus
+- Honest reporting, also when numbers are bad
+- Clear, short English
+SETUP
+- 10 hours per week to start, more when the account grows
+- $5 to $6 per hour depending on experience, paid weekly via Wise or PayPal
+- Long-term, ongoing
+- Flexible hours, one weekly call with the founder 
+- Tools: Seller Central, Amazon Ads console, Helium 10 (we provide access), Google Sheets, Slack or WhatsApp
+HOW TO APPLY
+1. Write "KAPSEL" as the first word of your application so we know you read this
+2. Send screenshots of 1 or 2 Amazon accounts you managed with ad spend, ACoS and sales visible
+3. Answer in 3 sentences: Amazon suppressed our best-selling listing because of a claim in the bullet points. What do you do in the first 24 hours, and what do you change so it does not happen again?
+Shortlisted candidates get a paid test task ($20, about 2 hours): a compliance and conversion audit of one of our listings on 
+ ---------- 
+ plus a PPC structure proposal.</t>
+        </is>
+      </c>
+      <c r="L357" s="4" t="inlineStr">
+        <is>
+          <t>We are a German dietary supplement brand (vitamins, minerals, capsules) selling on Amazon.de. The account is run by the founder, and we want one person who takes ownership of Amazon Germany: ads, listings, account health, and the rules that come…</t>
+        </is>
+      </c>
+      <c r="M357" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>1731809</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>Digital Relations Coordinator</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D358" s="3" t="inlineStr">
+        <is>
+          <t>PHP15,000 to 20,000/month</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="F358" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G358" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:35:10</t>
+        </is>
+      </c>
+      <c r="H358" s="4" t="inlineStr"/>
+      <c r="I358" s="4" t="inlineStr"/>
+      <c r="J358" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/digital-relations-coordinator-1731809</t>
+        </is>
+      </c>
+      <c r="K358" s="4" t="inlineStr">
+        <is>
+          <t>About the Role:
+Turn digital interactions into revenue as a Digital Relations Coordinator. You will spearhead high-velocity chat streams, command audience attention with magnetic copywriting, and transform active scrollers into loyal, paying buyers through dynamic text-based sales. 
+Schedule &amp; Work Arrangement: 
+100% remote flexibility allowing you to operate comfortably from your home office.
+ Dedicated 8-hour daily &amp; 5 to 7 days a week, synchronized with daytime hours in the Philippines.
+Shift schedules may occasionally shift to support changing operational coverage needs.
+What You’ll Earn:
+Guaranteed base salary amplified by lucrative daily performance incentives.
+Fast, secure, and hassle-free compensation delivered consistently via Wise.
+Full paid onboarding covering advanced messaging tactics and high-yielding sales strategies.
+Key Qualifications:
+Effortless mastery of current slang, casual idioms, and a smooth, conversational rhythm.
+Rapid typing performance (50+ WPM) designed to keep pace with high-volume digital chats.
+A dependable high-speed internet connection paired with a quiet, private home workspace.
+Pay Structure:
+Earn a base rate with commission and extra bonuses for daily results.</t>
+        </is>
+      </c>
+      <c r="L358" s="4" t="inlineStr">
+        <is>
+          <t>About the Role: Turn digital interactions into revenue as a Digital Relations Coordinator. You will spearhead high-velocity chat streams, command audience attention with magnetic copywriting, and transform active scrollers into loyal, paying buyers through dynamic text-based sales. Schedule &amp; Work…</t>
+        </is>
+      </c>
+      <c r="M358" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>1718668</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>Sales &amp; Customer Service Specialist</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D359" s="3" t="inlineStr">
+        <is>
+          <t>$600/mo</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="F359" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G359" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:32:51</t>
+        </is>
+      </c>
+      <c r="H359" s="4" t="inlineStr">
+        <is>
+          <t>Influencer Marketing, Shopify, Customer Service</t>
+        </is>
+      </c>
+      <c r="I359" s="4" t="inlineStr">
+        <is>
+          <t>Influencer Marketing, Shopify, Customer Service</t>
+        </is>
+      </c>
+      <c r="J359" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/sales-customer-service-specialist-1718668</t>
+        </is>
+      </c>
+      <c r="K359" s="4" t="inlineStr">
+        <is>
+          <t>Job Description
+We are looking for an experienced and motivated Sales &amp; Customer Service Specialist to join our team. The ideal candidate should have strong English communication skills, hands-on experience with Shopify or Shopline, and a background in sales and social media/influencer marketing.
+Key Responsibilities:
+Manage and operate Shopify or Shopline backend, including order processing, customer inquiries, and daily store operations.
+Product listing, Order fullfilment.
+Communicate with customers in English via email, phone, chat, and other communication channels.
+Respond to customer inquiries, provide product information, solve customer problems, and follow up on potential sales opportunities.
+Handle incoming inquiries and convert leads into orders through effective communication and sales skills.
+Build and maintain good relationships with customers and provide excellent customer service.
+Follow up with existing and potential customers to increase sales and customer retention.
+Assist with social media operations, including content posting and basic account management.
+Develop and contact social media influencers/content creators for potential collaborations.
+Maintain influencer contacts and follow up on collaboration opportunities.
+Requirements:
+1+ years of hands-on experience operating Shopify or Shopline backend.
+At least 2 years of sales or customer service experience; experience in e-commerce is a plus.
+Strong communication, customer service, and problem-solving skills.
+Experience with social media operations and influencer/KOL outreach.
+Experience developing influencers and establishing collaboration opportunities is preferred.
+Self-motivated, responsible, detail-oriented, and able to work independently.
+Preferred Qualifications:
+E-commerce experience, especially in home décor, lighting, furniture, or related industries.
+Experience working with international or U.S. customers.
+Familiarity with Instagram,
+ Facebook
+, TikTok, or other social media platforms.
+Experience using tools such as Shopify, Shopline, CRM systems, or other e-commerce platforms.
+Working Hours
+Monday–Saturday: 9:00 AM – 6:00 PM (U.S. Time)
+Sunday: Day Off
+（Please apply only if you are able to work the required schedule）</t>
+        </is>
+      </c>
+      <c r="L359" s="4" t="inlineStr">
+        <is>
+          <t>Job Description We are looking for an experienced and motivated Sales &amp; Customer Service Specialist to join our team. The ideal candidate should have strong English communication skills, hands-on experience with Shopify or Shopline, and a background in sales and…</t>
+        </is>
+      </c>
+      <c r="M359" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>1731805</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="inlineStr">
+        <is>
+          <t>Full Time Ecom Video Editor</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D360" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E360" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F360" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G360" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:31:54</t>
+        </is>
+      </c>
+      <c r="H360" s="4" t="inlineStr">
+        <is>
+          <t>Video Editing, AI Video Generation</t>
+        </is>
+      </c>
+      <c r="I360" s="4" t="inlineStr">
+        <is>
+          <t>Video Editing, AI Video Generation</t>
+        </is>
+      </c>
+      <c r="J360" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/full-time-ecom-video-editor-1731805</t>
+        </is>
+      </c>
+      <c r="K360" s="4" t="inlineStr">
+        <is>
+          <t>We’re looking for a talented Ecommerce Video Editor to join our team for a long term opportunity.
+What You’ll Be Editing:
+- Greenscreen/podcast/faceless style ads
+- UGC style ads
+What We’re Looking For:
+- Proven experience editing Ecommerce ads (please include examples)
+- Strong understanding of hooks, pacing, retention, and conversion driven storytelling
+- Ability to produce fast turnarounds
+- Full time availability
+- Someone who wants to grow long-term with a brand, not just freelance per project
+We value speed, creativity, and performance. If you’re hard working &amp; reliable, we’d love to hear from you.
+Please apply with your portfolio and a brief intro about your experience in ecom ad editing.
+‼️‼️‼️ PLEASE NOTE: DO NOT APPLY UNLESS YOU HAVE ECOMMERCE VIDEO EDITING EXPERIENCE.</t>
+        </is>
+      </c>
+      <c r="L360" s="4" t="inlineStr">
+        <is>
+          <t>We’re looking for a talented Ecommerce Video Editor to join our team for a long term opportunity. What You’ll Be Editing: - Greenscreen/podcast/faceless style ads - UGC style ads What We’re Looking For: - Proven experience editing Ecommerce ads (please…</t>
+        </is>
+      </c>
+      <c r="M360" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="inlineStr">
+        <is>
+          <t>1731803</t>
+        </is>
+      </c>
+      <c r="B361" s="3" t="inlineStr">
+        <is>
+          <t>Customer Support Agent</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D361" s="3" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="E361" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F361" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G361" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:28:14</t>
+        </is>
+      </c>
+      <c r="H361" s="4" t="inlineStr"/>
+      <c r="I361" s="4" t="inlineStr"/>
+      <c r="J361" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/customer-support-agent-1731803</t>
+        </is>
+      </c>
+      <c r="K361" s="4" t="inlineStr">
+        <is>
+          <t>We are looking for an English-speaking Customer Support Specialist with a strong service mindset and excellent communication skills. You’re the person who leaves customers smiling, whether it’s after a call, a chat, or an email.
+What you’ll do:
+As a Customer Support Specialist, you’re the first point of contact for our customers. You handle questions through various channels (phone, chat, email), and provide clear, helpful solutions.
+You’ll be fully trained on the subscriptions and services we offer, enabling you to confidently assist customers with a wide range of inquiries, from cancellations and refunds to other customer support-related questions.
+You’re also comfortable working with CRM systems and digital tools, we’ll show you the ropes!
+You're not just answering questions. You solve problems, think proactively, and help customers move forward.
+What we’re looking for
+Excellent English, both written and spoken
+At least 4/5 years of experience in customer support or a similar service role
+Strong communication skills – you can turn complex issues into clear answers
+Strong digital skills: familiar with CRM systems / different Platforms(e.g. Zoho, Olark and Aircall) and can quickly pick up new tools
+Detail-oriented 
+Problem-solver, you enjoy troubleshooting and finding the best solution
+Quick learner, you’re able to grasp new product and service information with ease
+Practical details:
+Full-time role: Working hours are Monday to Friday 9:00 - 18:00
+You have your own laptop and a stable internet connection
+You use a noise-canceling headset for clear communication
+Does this sound interesting? Please apply here and we're happy to jump in a call to discuss further.</t>
+        </is>
+      </c>
+      <c r="L361" s="4" t="inlineStr">
+        <is>
+          <t>We are looking for an English-speaking Customer Support Specialist with a strong service mindset and excellent communication skills. You’re the person who leaves customers smiling, whether it’s after a call, a chat, or an email. What you’ll do: As a…</t>
+        </is>
+      </c>
+      <c r="M361" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>1705924</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>Executive Assistant - Operations &amp; Follow-Through</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D362" s="3" t="inlineStr">
+        <is>
+          <t>$4-$6/hour</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F362" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G362" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:27:52</t>
+        </is>
+      </c>
+      <c r="H362" s="4" t="inlineStr">
+        <is>
+          <t>Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="I362" s="4" t="inlineStr">
+        <is>
+          <t>Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="J362" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/executive-assistant-operations-follow-through-1705924</t>
+        </is>
+      </c>
+      <c r="K362" s="4" t="inlineStr">
+        <is>
+          <t>DO NOT APPLY UNTIL YOU COMPLETE ALL 6 STEPS BELOW. Missing any one step means the application does not qualify.
+1. Complete the culture and job-fit interview: 
+ ---------- 
+2. Create one Google Doc and set access to anyone with the link can view.
+3. In the Doc, write CULTURE SCORE: followed by the score shown after the interview.
+4. In your own words, answer under these exact headings: WHAT I AM REALLY GOOD AT and WHAT I AM PASSIONATE ABOUT.
+5. In the Doc, write this exact confirmation: I did not use AI to write or rewrite these answers.
+6. Submit one OnlineJobs application that starts with ANCHOR, includes the public Google Doc link, and ends with COMPLETE.
+Check your Doc in an incognito/private browser before applying. If we message you about a missing item, update the same Doc and reply once all 6 steps are complete. We only review applications after all 6 steps are verified.
+We need a full-time Executive Assistant who reads SOPs carefully, solves routine problems, and closes every assigned item without constant reminders.
+The work includes hiring support, research, documentation, scheduling, account setup, profile updates, source checking, approved support drafts, and follow-up. Every task must finish as done, blocked with evidence, or explicitly deferred.
+After the Google Doc link, use these exact labels:
+- Detail example: one prior task where small instructions mattered and how you verified every step.
+- Blocker example: one real blocker you solved before escalating, including what you tried.
+- Follow-through example: one prior task that required repeated follow-up until completion.
+- Initiative example: one useful risk or adjacent task you noticed and proposed without overstepping your access.
+- Rate: your hourly rate.
+- Availability: weekly hours and timezone.
+Do not perform live work, contact anyone, or create a production deliverable for this application. The Google Doc is a short self-reflection, not a work assignment.
+The final stage is a paid 3-day trial. Before it starts, we will state the exact tasks, output count, deadline, quality bar, communication cadence, and pass standard. The trial will test SOP accuracy, problem solving, useful questions, initiative, capacity, and complete follow-through. We proceed only when the result is a clear yes.</t>
+        </is>
+      </c>
+      <c r="L362" s="4" t="inlineStr">
+        <is>
+          <t>DO NOT APPLY UNTIL YOU COMPLETE ALL 6 STEPS BELOW. Missing any one step means the application does not qualify. 1. Complete the culture and job-fit interview: https://ugc.gobuildfast.com/quiz 2. Create one Google Doc and set access to anyone with the…</t>
+        </is>
+      </c>
+      <c r="M362" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>1731801</t>
+        </is>
+      </c>
+      <c r="B363" s="3" t="inlineStr">
+        <is>
+          <t>Google Ads Performance Analyst</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D363" s="3" t="inlineStr">
+        <is>
+          <t>$1200-1500/month</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F363" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G363" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:26:56</t>
+        </is>
+      </c>
+      <c r="H363" s="4" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="I363" s="4" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="J363" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/google-ads-performance-analyst-1731801</t>
+        </is>
+      </c>
+      <c r="K363" s="4" t="inlineStr">
+        <is>
+          <t>We spend across several Google accounts and our reporting does not currently tell us much. We want that fixed.
+Day to day: Tracking cost per conversion, conversion rate, and return on ad spend across accounts. Checking that conversion tracking is set up correctly and firing as expected. Comparing performance across campaign types to see where budget is best placed. Maintaining reporting sheets or dashboards. Writing up what changed and what it means.
+What we need: Genuine comfort with numbers. Understanding of Google Ads conversion tracking and how conversions are counted. Pivot tables and formulas as routine work. Ability to explain a finding in plain writing.
+Nice to have: Google Analytics 4. Looker Studio. Understanding of attribution models and why two reports can disagree.
+The person we are looking for: Someone who questions a number that looks too good before passing it on. We would rather hear the caveat early.
+To apply, send your CV to:
+jermainenunez2796 gmail com</t>
+        </is>
+      </c>
+      <c r="L363" s="4" t="inlineStr">
+        <is>
+          <t>We spend across several Google accounts and our reporting does not currently tell us much. We want that fixed. Day to day: Tracking cost per conversion, conversion rate, and return on ad spend across accounts. Checking that conversion tracking is…</t>
+        </is>
+      </c>
+      <c r="M363" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>1731800</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>PPC Campaign Assistant</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="inlineStr">
+        <is>
+          <t>$1200-1500/month</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F364" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G364" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:26:36</t>
+        </is>
+      </c>
+      <c r="H364" s="4" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="I364" s="4" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="J364" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/ppc-campaign-assistant-1731800</t>
+        </is>
+      </c>
+      <c r="K364" s="4" t="inlineStr">
+        <is>
+          <t>Campaign building and account housekeeping take more time than they should. We want one person owning that work properly.
+Day to day: Building out campaigns, ad groups, and keyword lists from briefs. Writing headline and description variations for responsive search ads. Setting up and checking ad extensions. Keeping naming conventions consistent across the account. Checking landing page links before anything goes live.
+What we need: Familiarity with the Google Ads interface and how campaigns are structured. Readable written English, since ad copy is part of this. Careful attention to detail. Google Sheets for keyword and build sheets.
+Nice to have: Google Ads Editor. Basic keyword research using Keyword Planner.
+The person we are looking for: Someone who double-checks a URL before publishing. Small errors here cost real money, and we notice when someone prevents them.
+To apply, send your CV to:
+jermainenunez2796 gmail com</t>
+        </is>
+      </c>
+      <c r="L364" s="4" t="inlineStr">
+        <is>
+          <t>Campaign building and account housekeeping take more time than they should. We want one person owning that work properly. Day to day: Building out campaigns, ad groups, and keyword lists from briefs. Writing headline and description variations for responsive search…</t>
+        </is>
+      </c>
+      <c r="M364" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>1731799</t>
+        </is>
+      </c>
+      <c r="B365" s="3" t="inlineStr">
+        <is>
+          <t>Google Ads Manager - Search and Shopping</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D365" s="3" t="inlineStr">
+        <is>
+          <t>$1200-1500/month</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F365" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G365" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:26:19</t>
+        </is>
+      </c>
+      <c r="H365" s="4" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="I365" s="4" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="J365" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/google-ads-manager-search-and-shopping-1731799</t>
+        </is>
+      </c>
+      <c r="K365" s="4" t="inlineStr">
+        <is>
+          <t>Our Google account has been running on autopilot longer than it should have. We want someone to take it back in hand.
+Day to day: Managing Search and Shopping campaigns day to day. Reviewing search terms and adding negatives so budget stops going to irrelevant clicks. Adjusting bids and budgets based on what is converting. Keeping ad groups tight rather than letting them sprawl. Writing and rotating responsive search ad assets.
+What we need: Working comfort inside Google Ads. Understanding of keyword match types and why the search terms report matters. Ability to read conversion data and act on it. Spreadsheet fluency. Clear written English for updates.
+Nice to have: Shopping feed or Merchant Center exposure. Familiarity with Performance Max.
+The person we are looking for: Someone who reviews search terms because they want to see what is leaking, not because it is scheduled. That habit alone pays for the role.
+To apply, send your CV to:
+jermainenunez2796 gmail com</t>
+        </is>
+      </c>
+      <c r="L365" s="4" t="inlineStr">
+        <is>
+          <t>Our Google account has been running on autopilot longer than it should have. We want someone to take it back in hand. Day to day: Managing Search and Shopping campaigns day to day. Reviewing search terms and adding negatives so…</t>
+        </is>
+      </c>
+      <c r="M365" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>1731798</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>Performance Analyst - Meta Advertising</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D366" s="3" t="inlineStr">
+        <is>
+          <t>$1200-1500/month</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F366" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G366" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:25:47</t>
+        </is>
+      </c>
+      <c r="H366" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="I366" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="J366" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/performance-analyst-meta-advertising-1731798</t>
+        </is>
+      </c>
+      <c r="K366" s="4" t="inlineStr">
+        <is>
+          <t>We would rather know the real number than the flattering one. That is what this role is for.
+Day to day: Tracking cost per acquisition, conversion rate, and return on ad spend. Identifying where the funnel drops off. Verifying the pixel is firing the events we assume it is. Keeping dashboards current. Reporting findings honestly, including the ones nobody wants.
+What we need: Genuine comfort with numbers. Familiarity with the Meta Pixel and standard conversion events. Pivot tables and formulas as routine work. Ability to explain a finding in writing, not just hand over a sheet.
+Nice to have: Google Analytics or similar. Understanding of UTM parameters.
+The person we are looking for: Someone willing to say a campaign is not working while it is still running. Diplomatically, but clearly.
+To apply, send your CV to:
+jermainenunez2796 gmail com</t>
+        </is>
+      </c>
+      <c r="L366" s="4" t="inlineStr">
+        <is>
+          <t>We would rather know the real number than the flattering one. That is what this role is for. Day to day: Tracking cost per acquisition, conversion rate, and return on ad spend. Identifying where the funnel drops off. Verifying the…</t>
+        </is>
+      </c>
+      <c r="M366" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>1731796</t>
+        </is>
+      </c>
+      <c r="B367" s="3" t="inlineStr">
+        <is>
+          <t>Business Manager Administrator</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="D367" s="3" t="inlineStr">
+        <is>
+          <t>$15-50/hour</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F367" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G367" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:25:20</t>
+        </is>
+      </c>
+      <c r="H367" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="I367" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="J367" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/business-manager-administrator-1731796</t>
+        </is>
+      </c>
+      <c r="K367" s="4" t="inlineStr">
+        <is>
+          <t>An administrative role for someone who takes satisfaction in records being correct and complete.
+Day to day: Setting up and maintaining Business Manager assets — pages, pixels, ad accounts. Managing access: granting roles, removing them promptly when someone leaves, keeping permissions at the right level. Keeping billing details accurate. Maintaining the master record of what exists and who can reach it.
+What we need: Understanding of how Business Manager is structured and what each permission level actually permits. Willingness to follow documented procedure rather than shortcuts. Written English clear enough for the team to follow your notes.
+Nice to have: Two-factor authentication and general account security practice. Comfort working across several portfolios.
+The person we are looking for: Someone who would rather ask than assume when a request is ambiguous. All administration follows Meta's platform requirements, and we train step by step before handing anything over. Part-time hours agreed together.
+To apply, send your CV to:
+jermainenunez2796 gmail com</t>
+        </is>
+      </c>
+      <c r="L367" s="4" t="inlineStr">
+        <is>
+          <t>An administrative role for someone who takes satisfaction in records being correct and complete. Day to day: Setting up and maintaining Business Manager assets — pages, pixels, ad accounts. Managing access: granting roles, removing them promptly when someone leaves, keeping…</t>
+        </is>
+      </c>
+      <c r="M367" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>1731795</t>
+        </is>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>Paid Social Ads Assistant</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D368" s="3" t="inlineStr">
+        <is>
+          <t>$1200-1500/month</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F368" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G368" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:24:39</t>
+        </is>
+      </c>
+      <c r="H368" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="I368" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="J368" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/paid-social-ads-assistant-1731795</t>
+        </is>
+      </c>
+      <c r="K368" s="4" t="inlineStr">
+        <is>
+          <t>We lose more time to badly built ad sets than to bad ideas. This role is about building them properly.
+Day to day: Setting up ad sets and loading copy and creative. Requesting the assets you need from the designer or editor rather than making do. Keeping naming and folder structure consistent so the account is still readable months later. Recording which variation came out ahead and why.
+What we need: Ability to build audiences in Ads Manager on your own, custom and lookalike included. Readable written English, since you will be handling copy. A natural tendency to organize.
+Nice to have: Canva or basic image editing. Comfort with Reels and vertical formats.
+The person we are looking for: Someone who is bothered by disorder. If an untidy account makes you want to fix it, you will do well here.
+To apply, send your CV to:
+jermainenunez2796 gmail com</t>
+        </is>
+      </c>
+      <c r="L368" s="4" t="inlineStr">
+        <is>
+          <t>We lose more time to badly built ad sets than to bad ideas. This role is about building them properly. Day to day: Setting up ad sets and loading copy and creative. Requesting the assets you need from the designer…</t>
+        </is>
+      </c>
+      <c r="M368" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
+          <t>1725875</t>
+        </is>
+      </c>
+      <c r="B369" s="3" t="inlineStr">
+        <is>
+          <t>Process Support Specialist (Remote)</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D369" s="3" t="inlineStr">
+        <is>
+          <t>PHP 30,000 - PHP 40,000</t>
+        </is>
+      </c>
+      <c r="E369" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F369" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G369" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:24:25</t>
+        </is>
+      </c>
+      <c r="H369" s="4" t="inlineStr">
+        <is>
+          <t>Construction And Engineering, Administrative Management, Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="I369" s="4" t="inlineStr">
+        <is>
+          <t>Construction And Engineering, Administrative Management, Virtual Assistant</t>
+        </is>
+      </c>
+      <c r="J369" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/process-support-specialist-remote-1725875</t>
+        </is>
+      </c>
+      <c r="K369" s="4" t="inlineStr">
+        <is>
+          <t>About the Role
+We are looking for a detail-oriented, proactive Process Support Specialist to assist our HVAC operations. You will serve as the backbone of day-to-day administration, ensuring warranty registrations, invoices, customer follow-ups, and operational workflow run seamlessly.
+Key Responsibilities
+Prepare, process, and audit customer invoices with high accuracy.
+Submit and track manufacturer warranty registrations and rebate documentation.
+Maintain clean digital records, CRM database entries, and job files.
+Provide operations support to field team managers and assist with essential customer service duties.
+Create and schedule basic social media posts to keep the local community engaged.
+What We’re Looking For
+Trade/Service Industry Experience (Required): Prior background supporting HVAC, plumbing, electrical, or general trade contractors.
+Administrative Expertise: Proven track record as a Virtual Assistant, Admin Specialist, or Operations Assistant in a remote setting.
+Documentation Savvy: Hands-on experience navigating permits, trade rebates, or warranty claims processes.
+Tech-Minded: Comfortable using modern CRMs, project management platforms, and AI efficiency tools.
+Communication: Exceptional written and verbal English skills.
+How to Apply
+Ready to elevate your virtual assistant career? Click "Apply for this Job" and include:
+A brief 2-3 sentence summary of your experience with HVAC or trade-service businesses.
+A link to your updated resume (Google Drive or Dropbox set to public access).
+The word ASAP as your subject title.</t>
+        </is>
+      </c>
+      <c r="L369" s="4" t="inlineStr">
+        <is>
+          <t>About the Role We are looking for a detail-oriented, proactive Process Support Specialist to assist our HVAC operations. You will serve as the backbone of day-to-day administration, ensuring warranty registrations, invoices, customer follow-ups, and operational workflow run seamlessly. Key Responsibilities…</t>
+        </is>
+      </c>
+      <c r="M369" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="inlineStr">
+        <is>
+          <t>1731794</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>Media Buyer - Meta Ads</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="D370" s="3" t="inlineStr">
+        <is>
+          <t>$1200-1500/month</t>
+        </is>
+      </c>
+      <c r="E370" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F370" s="3" t="inlineStr">
+        <is>
+          <t>Sep 16, 2026</t>
+        </is>
+      </c>
+      <c r="G370" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 15:24:19</t>
+        </is>
+      </c>
+      <c r="H370" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="I370" s="4" t="inlineStr">
+        <is>
+          <t>Facebook marketing, Facebook Ads</t>
+        </is>
+      </c>
+      <c r="J370" s="5" t="inlineStr">
+        <is>
+          <t>https://www.onlinejobs.ph/jobseekers/job/media-buyer-meta-ads-1731794</t>
+        </is>
+      </c>
+      <c r="K370" s="4" t="inlineStr">
+        <is>
+          <t>Someone needs to be the person who notices when a campaign starts slipping. Right now nobody owns that consistently.
+Day to day: Reviewing accounts each morning and acting on what you find. Cutting spend that has stopped producing. Reallocating toward what is holding. Queuing the next round of tests before the current set goes flat. Recording what you changed and your reasoning, so decisions can be reviewed later.
+What we need: Working comfort in Ads Manager. The ability to look at a performance breakdown and form a view rather than waiting to be told. Spreadsheet fluency. English clear enough for a short written update.
+Nice to have: E-commerce or lead gen exposure. Any structured habit around testing.
+The person we are looking for: Someone who checks the account because they want to know, not because it is on a checklist. That instinct is the thing we cannot train.
+To apply, send your CV to:
+jermainenunez2796 gmail com</t>
+        </is>
+      </c>
+      <c r="L370" s="4" t="inlineStr">
+        <is>
+          <t>Someone needs to be the person who notices when a campaign starts slipping. Right now nobody owns that consistently. Day to day: Reviewing accounts each morning and acting on what you find. Cutting spend that has stopped producing. Reallocating toward…</t>
+        </is>
+      </c>
+      <c r="M370" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:54:28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M350"/>
+  <autoFilter ref="A1:M370"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -37983,6 +39704,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J348" r:id="rId347"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J349" r:id="rId348"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J370" r:id="rId369"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>